<commit_message>
SVO Match Engine v1.0 production
</commit_message>
<xml_diff>
--- a/output/ARRIVAL_MATCH_None.xlsx
+++ b/output/ARRIVAL_MATCH_None.xlsx
@@ -1483,19 +1483,23 @@
       <c r="K20" s="4" t="n"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>SKU-064</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Кондиционер SVO Lotos 2,7 л</t>
+        </is>
+      </c>
       <c r="O20" t="n">
-        <v>64.25</v>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>MULTIPLE_MATCH,LOW_SCORE,NO_VOLUME</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -7481,19 +7485,23 @@
       <c r="K175" s="4" t="n"/>
       <c r="L175" t="inlineStr">
         <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="M175" t="inlineStr"/>
-      <c r="N175" t="inlineStr"/>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>SKU-283</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>Подгузники BOSSFIX Size 1 1 уп</t>
+        </is>
+      </c>
       <c r="O175" t="n">
-        <v>45</v>
-      </c>
-      <c r="P175" t="inlineStr">
-        <is>
-          <t>MULTIPLE_MATCH,LOW_SCORE,NO_VOLUME</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="P175" t="inlineStr"/>
     </row>
     <row r="176" ht="6.75" customHeight="1" s="15">
       <c r="A176" s="3" t="inlineStr">
@@ -10147,7 +10155,7 @@
       </c>
       <c r="N240" t="inlineStr">
         <is>
-          <t>Кофе зерно Yunis Effendi  500 г</t>
+          <t>Кофе зерно Yunis Effendi 500 г</t>
         </is>
       </c>
       <c r="O240" t="n">
@@ -10185,7 +10193,7 @@
       </c>
       <c r="N241" t="inlineStr">
         <is>
-          <t>Кофе молотый Yunis Effendi  100 г</t>
+          <t>Кофе молотый Yunis Effendi 100 г</t>
         </is>
       </c>
       <c r="O241" t="n">
@@ -10223,7 +10231,7 @@
       </c>
       <c r="N242" t="inlineStr">
         <is>
-          <t>Кофе молотый Yunis Effendi  250 г</t>
+          <t>Кофе молотый Yunis Effendi 250 г</t>
         </is>
       </c>
       <c r="O242" t="n">
@@ -11187,7 +11195,7 @@
       </c>
       <c r="N267" t="inlineStr">
         <is>
-          <t>Антинакипь DOMIX  1 л</t>
+          <t>Антинакипь DOMIX 1 л</t>
         </is>
       </c>
       <c r="O267" t="n">
@@ -11227,7 +11235,7 @@
       </c>
       <c r="N268" t="inlineStr">
         <is>
-          <t>Антижир DOMIX  1 л</t>
+          <t>Антижир DOMIX 1 л</t>
         </is>
       </c>
       <c r="O268" t="n">

</xml_diff>